<commit_message>
Merge live OTA channel price samples into Magenta Excel report.
Adds Booking/Airbnb/Rentalia/HomeToGo readings across 1–3 night dates, marks Expedia/VRBO/MagentaStay failures, and includes raw JSON plus summary for the Sanchioli 11 channel check.

Co-authored-by: fabio <fabiopulina@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LocazioneTuristica/report-prezzi-magenta-competitor.xlsx
+++ b/LocazioneTuristica/report-prezzi-magenta-competitor.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Riepilogo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tuoi canali" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Competitor Magenta" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Per scenario" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Note metodo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Confronto canali" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Competitor Magenta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Per scenario" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Note metodo" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,7 +50,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -114,6 +120,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1179,1316 +1186,1855 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Prezzi Sanchioli 11 sui tuoi canali (campioni)</t>
+          <t>Prezzi Sanchioli 11 — campionamento live sui tuoi canali</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Booking = live search Magenta 27 ott 2026 · MagentaStay = listino AvaiBook · altri = da verificare / captcha</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+          <t>Fonte: browser scrape 27 ott 2026 (Europe/Rome) · 2 adulti · dati da Sample OTA prices multi-night</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Booking/Airbnb/Rentalia/HomeToGo live dove possibile; Expedia/VRBO spesso bloccati; MagentaStay widget errore date</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Check-in</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Check-out</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Notti</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Canale</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>€/notte</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Totale €</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Stato</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>MagentaStay</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>MagentaStay</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>95</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>190</v>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>stimato AvaiBook</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>https://www.magentastay.it/strutture/sanchioli-11/</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>AvaiBook base stimato</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>widget validation error - delegates to AvaiBook</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>errore</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>282</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>258</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>86</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>113</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>113</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Booking</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
+      <c r="E13" s="6" t="n">
+        <v>157</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>143</v>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>144</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/sanchioli.it.html</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>A notte€ 72</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>2027-02-06</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>2027-02-08</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>248</v>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>2027-02-06</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>2027-02-08</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-14</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-17</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-14</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-17</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>398</v>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>132.67</v>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>non-refundable</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="n"/>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>305</v>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>152.5</v>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation until Oct 31</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D27" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>parziale</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.airbnb.it/rooms/1780316664494400682</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>218 € in totale
-Mostra il dettaglio dei prezzi
-218 € in totale
-CHECK-IN
-10/11/2026
-CHECK-OUT
-12/11</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>not tested in this session</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>2027-02-06</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>2027-02-08</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>262</v>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>131</v>
+      </c>
+      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-14</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>2027-04-17</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>457</v>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>152.33</v>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="n"/>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>error - date validation failed</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>errore</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D34" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>MagentaStay</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>147.5</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>295</v>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>stimato AvaiBook</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.magentastay.it/strutture/sanchioli-11/</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>AvaiBook base stimato</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>EICMA weekend</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>189</v>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>error - date validation failed</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>errore</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="n"/>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I38" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>2027-02-06</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>2027-02-08</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="n"/>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-14</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-17</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="n"/>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I40" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="n"/>
+      <c r="H41" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I41" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I42" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D43" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Booking</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>102</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>204</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/sanchioli.it.html</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>A notte€ 102</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="n"/>
+      <c r="H43" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I43" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>2026-11-07</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="n"/>
+      <c r="H44" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I44" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Airbnb</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>parziale</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.airbnb.it/rooms/1780316664494400682</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>305 € in totale
-Mostra il dettaglio dei prezzi
-305 € in totale
-CHECK-IN
-05/11/2026
-CHECK-OUT
-07/11</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="E45" s="6" t="n">
+        <v>260.96</v>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>prices in USD</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>2026-11-11</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C46" s="10" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D46" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>MagentaStay</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>95</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>95</v>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>stimato AvaiBook</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.magentastay.it/strutture/sanchioli-11/</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>AvaiBook base stimato</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="n"/>
+      <c r="H46" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I46" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="10" t="n"/>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="n"/>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>2027-02-06</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>2027-02-08</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="10" t="n"/>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="n"/>
+      <c r="H48" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-14</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-17</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="10" t="n"/>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="n"/>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>not tested</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
+        <is>
+          <t>mancante</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Expedia</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Booking</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>72</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>72</v>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/sanchioli.it.html</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>A notte€ 72</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="D50" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>blocked - bot detection</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>bloccato</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>VRBO</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Airbnb</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>parziale</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>https://www.airbnb.it/rooms/1780316664494400682</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>109 € in totale
-Mostra il dettaglio dei prezzi
-109 € in totale
-CHECK-IN
-11/11/2026
-CHECK-OUT
-12/11</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>MagentaStay</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>146.67</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>440</v>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>stimato AvaiBook</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>https://www.magentastay.it/strutture/sanchioli-11/</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>AvaiBook base stimato</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Booking</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>101</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>303</v>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/sanchioli.it.html</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>A notte€ 101</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Airbnb</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>parziale</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.airbnb.it/rooms/1780316664494400682</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>454 € in totale
-Mostra il dettaglio dei prezzi
-454 € in totale
-CHECK-IN
-04/11/2026
-CHECK-OUT
-07/11</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="n">
+      <c r="D51" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Rentalia</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>https://it.rentalia.com/1043251</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>da campionare live</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>HomeToGo</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hometogo.it/rental/425c00291ea2ccb1</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>spesso Cloudflare</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Expedia</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>https://www.expedia.com/Milan-Hotels-Studio-Apartment-In-Magenta-Near-Rho-Fiera.h136647276.Hotel-Information</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>captcha frequente</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>midweek</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>VRBO</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vrbo.com/it-it/affitto-vacanze/p12260884</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>captcha / sync manuale</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Rentalia</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>https://it.rentalia.com/1043251</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>da campionare live</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>HomeToGo</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hometogo.it/rental/425c00291ea2ccb1</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>spesso Cloudflare</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Expedia</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>https://www.expedia.com/Milan-Hotels-Studio-Apartment-In-Magenta-Near-Rho-Fiera.h136647276.Hotel-Information</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>captcha frequente</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>eicma</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>VRBO</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vrbo.com/it-it/affitto-vacanze/p12260884</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>captcha / sync manuale</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Rentalia</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>https://it.rentalia.com/1043251</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>da campionare live</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>HomeToGo</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hometogo.it/rental/425c00291ea2ccb1</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>spesso Cloudflare</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Expedia</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>https://www.expedia.com/Milan-Hotels-Studio-Apartment-In-Magenta-Near-Rho-Fiera.h136647276.Hotel-Information</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>captcha frequente</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>1night</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>VRBO</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vrbo.com/it-it/affitto-vacanze/p12260884</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>captcha / sync manuale</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Rentalia</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>https://it.rentalia.com/1043251</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>da campionare live</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>HomeToGo</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hometogo.it/rental/425c00291ea2ccb1</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>spesso Cloudflare</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Expedia</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>https://www.expedia.com/Milan-Hotels-Studio-Apartment-In-Magenta-Near-Rho-Fiera.h136647276.Hotel-Information</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>captcha frequente</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>3night_eicma</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>2026-11-07</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>VRBO</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vrbo.com/it-it/affitto-vacanze/p12260884</t>
-        </is>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>captcha / sync manuale</t>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="n"/>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>page loading issue - pricing widget not visible</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>errore</t>
         </is>
       </c>
     </row>
@@ -2498,6 +3044,668 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Confronto €/notte Sanchioli 11 tra canali (solo letture OK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29 → 2026-11-01 (3 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>282</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Min Booking 86.0 €/n · Max Booking 94.0 €/n · spread 8.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-05 → 2026-11-07 (2 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>305</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>152.5</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation until Oct 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Min Airbnb 152.5 €/n · Max Airbnb 152.5 €/n · spread 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07 → 2026-11-08 (1 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>113</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>113</v>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>EICMA weekend</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Min Booking 104.0 €/n · Max Rentalia 126.0 €/n · spread 22.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-10 → 2026-11-12 (2 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>157</v>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Rentalia</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>189</v>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>HomeToGo</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>260.96</v>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>prices in USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Min Booking 71.5 €/n · Max HomeToGo 120.0 €/n · spread 48.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-11 → 2026-11-12 (1 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Min Booking 72.0 €/n · Max Booking 78.0 €/n · spread 6.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-12-10 → 2026-12-11 (1 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="E39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Min Booking 84.0 €/n · Max Airbnb 126.0 €/n · spread 42.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>2027-02-06 → 2027-02-08 (2 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>248</v>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="n">
+        <v>262</v>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>131</v>
+      </c>
+      <c r="E46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Min Booking 113.5 €/n · Max Airbnb 131.0 €/n · spread 17.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>2027-04-14 → 2027-04-17 (3 notti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Canale</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Totale</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Valuta</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>€/notte</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Booking</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n">
+        <v>435</v>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>free cancellation</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>457</v>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>152.33</v>
+      </c>
+      <c r="E53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Min Booking 132.7 €/n · Max Airbnb 152.3 €/n · spread 19.7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9152,7 +10360,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12542,13 +13750,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12622,6 +13830,34 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Aggiornamento canali propri: sample browser (Booking, Airbnb, Rentalia, HomeToGo, Expedia, VRBO, MagentaStay).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Expedia spesso "blocked"; VRBO widget prezzi non renderizza; MagentaStay errore validazione date widget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>JSON grezzo: /opt/cursor/artifacts/ota-prices/ota-canali-sample.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Summary MD: /opt/cursor/artifacts/ota-canali-sample-summary.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>